<commit_message>
funktionierende seite vor strukturanpassung
</commit_message>
<xml_diff>
--- a/outputs/struktur-georgien-2026/georgien-2026-inhaltsstruktur.xlsx
+++ b/outputs/struktur-georgien-2026/georgien-2026-inhaltsstruktur.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Arbeitsnotizen (vorher)" sheetId="1" r:id="Rb18eaf55b0464b0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ergänzen &amp; prüfen" sheetId="2" r:id="Rd5adcb5a43274872"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seitenregister" sheetId="3" r:id="R53ee9310262f457a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Arbeitsnotizen (vorher)" sheetId="1" r:id="R50494a79a0f0499c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ergänzen &amp; prüfen" sheetId="2" r:id="R5fbb8801663244da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seitenregister" sheetId="3" r:id="Rc4db0d1a35b94460"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -973,7 +973,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="39">
+  <x:cellXfs count="40">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
@@ -1075,6 +1075,9 @@
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
     <x:cellStyle name="Normal" xfId="1"/>
@@ -1175,7 +1178,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SeitenregisterTable" displayName="SeitenregisterTable" ref="A4:J160" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SeitenregisterTable" displayName="SeitenregisterTable" ref="A4:J178" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Abschnitt"/>
     <x:tableColumn id="2" name="Kapitel"/>
@@ -3285,7 +3288,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R67ce365c61624778"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rece963db28744ce5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3433,7 +3436,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb63755d31a9f4263"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06c90bf3d39c4f80"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7168,7 +7171,7 @@
         <x:v>Ja</x:v>
       </x:c>
       <x:c r="I121" s="33" t="str">
-        <x:v>Vorhandenes Bild prüfen</x:v>
+        <x:v>Adscharisches Chatschapuri hier integrieren; bisherige Detail-URL später auf diese Seite weiterleiten.</x:v>
       </x:c>
       <x:c r="J121" s="33" t="str">
         <x:v>Kachel / Link bei Kulinarik</x:v>
@@ -8338,6 +8341,582 @@
       <x:c r="I160" s="34" t="str"/>
       <x:c r="J160" s="34" t="str">
         <x:v>Technisch / kein Menü</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="161">
+      <x:c r="A161" s="30" t="str">
+        <x:v>Essen &amp; Trinken</x:v>
+      </x:c>
+      <x:c r="B161" s="30" t="str">
+        <x:v>Restaurants</x:v>
+      </x:c>
+      <x:c r="C161" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D161" s="30" t="str">
+        <x:v>360 Sky Bar</x:v>
+      </x:c>
+      <x:c r="E161" s="39" t="n">
+        <x:v>157</x:v>
+      </x:c>
+      <x:c r="F161" s="30" t="str">
+        <x:v>13.2</x:v>
+      </x:c>
+      <x:c r="G161" s="30" t="str">
+        <x:v>Eigene Restaurantseite mit Atmosphäre, Angebot, Lage, Reservationshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H161" s="30" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="I161" s="30" t="str">
+        <x:v>Vorhandenes Bild prüfen</x:v>
+      </x:c>
+      <x:c r="J161" s="30" t="str">
+        <x:v>Kachel / Link bei Restaurants</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="162">
+      <x:c r="A162" s="30" t="str">
+        <x:v>Essen &amp; Trinken</x:v>
+      </x:c>
+      <x:c r="B162" s="30" t="str">
+        <x:v>Restaurants</x:v>
+      </x:c>
+      <x:c r="C162" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D162" s="30" t="str">
+        <x:v>Baia’s Wine</x:v>
+      </x:c>
+      <x:c r="E162" s="39" t="n">
+        <x:v>158</x:v>
+      </x:c>
+      <x:c r="F162" s="30" t="str">
+        <x:v>13.2</x:v>
+      </x:c>
+      <x:c r="G162" s="30" t="str">
+        <x:v>Eigene Restaurantseite mit Atmosphäre, Angebot, Lage, Reservationshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H162" s="30" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="I162" s="30" t="str">
+        <x:v>Vorhandenes Bild prüfen</x:v>
+      </x:c>
+      <x:c r="J162" s="30" t="str">
+        <x:v>Kachel / Link bei Restaurants</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="163">
+      <x:c r="A163" s="30" t="str">
+        <x:v>Essen &amp; Trinken</x:v>
+      </x:c>
+      <x:c r="B163" s="30" t="str">
+        <x:v>Restaurants</x:v>
+      </x:c>
+      <x:c r="C163" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D163" s="30" t="str">
+        <x:v>Barbarestan</x:v>
+      </x:c>
+      <x:c r="E163" s="39" t="n">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="F163" s="30" t="str">
+        <x:v>13.2</x:v>
+      </x:c>
+      <x:c r="G163" s="30" t="str">
+        <x:v>Eigene Restaurantseite mit Atmosphäre, Angebot, Lage, Reservationshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H163" s="30" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="I163" s="30" t="str">
+        <x:v>Vorhandenes Bild prüfen</x:v>
+      </x:c>
+      <x:c r="J163" s="30" t="str">
+        <x:v>Kachel / Link bei Restaurants</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="164">
+      <x:c r="A164" s="30" t="str">
+        <x:v>Essen &amp; Trinken</x:v>
+      </x:c>
+      <x:c r="B164" s="30" t="str">
+        <x:v>Restaurants</x:v>
+      </x:c>
+      <x:c r="C164" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D164" s="30" t="str">
+        <x:v>Keto &amp; Kote</x:v>
+      </x:c>
+      <x:c r="E164" s="39" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="F164" s="30" t="str">
+        <x:v>13.2</x:v>
+      </x:c>
+      <x:c r="G164" s="30" t="str">
+        <x:v>Eigene Restaurantseite mit Atmosphäre, Angebot, Lage, Reservationshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H164" s="30" t="str">
+        <x:v>Ja</x:v>
+      </x:c>
+      <x:c r="I164" s="30" t="str">
+        <x:v>Vorhandenes Bild prüfen</x:v>
+      </x:c>
+      <x:c r="J164" s="30" t="str">
+        <x:v>Kachel / Link bei Restaurants</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="165">
+      <x:c r="A165" s="30" t="str">
+        <x:v>Essen &amp; Trinken</x:v>
+      </x:c>
+      <x:c r="B165" s="30" t="str">
+        <x:v>Restaurants</x:v>
+      </x:c>
+      <x:c r="C165" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D165" s="30" t="str">
+        <x:v>Laguna</x:v>
+      </x:c>
+      <x:c r="E165" s="39" t="n">
+        <x:v>161</x:v>
+      </x:c>
+      <x:c r="F165" s="30" t="str">
+        <x:v>13.2</x:v>
+      </x:c>
+      <x:c r="G165" s="30" t="str">
+        <x:v>Eigene Restaurantseite mit Atmosphäre, Angebot, Lage, Reservationshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H165" s="30" t="str">
+        <x:v>Platzhalter</x:v>
+      </x:c>
+      <x:c r="I165" s="30" t="str">
+        <x:v>platzhalter.png, bis ein lizenziertes Bild vorliegt</x:v>
+      </x:c>
+      <x:c r="J165" s="30" t="str">
+        <x:v>Kachel / Link bei Restaurants</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="166">
+      <x:c r="A166" s="30" t="str">
+        <x:v>Essen &amp; Trinken</x:v>
+      </x:c>
+      <x:c r="B166" s="30" t="str">
+        <x:v>Restaurants</x:v>
+      </x:c>
+      <x:c r="C166" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D166" s="30" t="str">
+        <x:v>Palaty</x:v>
+      </x:c>
+      <x:c r="E166" s="39" t="n">
+        <x:v>162</x:v>
+      </x:c>
+      <x:c r="F166" s="30" t="str">
+        <x:v>13.2</x:v>
+      </x:c>
+      <x:c r="G166" s="30" t="str">
+        <x:v>Eigene Restaurantseite mit Atmosphäre, Angebot, Lage, Reservationshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H166" s="30" t="str">
+        <x:v>Platzhalter</x:v>
+      </x:c>
+      <x:c r="I166" s="30" t="str">
+        <x:v>platzhalter.png, bis ein lizenziertes Bild vorliegt</x:v>
+      </x:c>
+      <x:c r="J166" s="30" t="str">
+        <x:v>Kachel / Link bei Restaurants</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="167">
+      <x:c r="A167" s="30" t="str">
+        <x:v>Essen &amp; Trinken</x:v>
+      </x:c>
+      <x:c r="B167" s="30" t="str">
+        <x:v>Restaurants</x:v>
+      </x:c>
+      <x:c r="C167" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D167" s="30" t="str">
+        <x:v>Pasanauri</x:v>
+      </x:c>
+      <x:c r="E167" s="39" t="n">
+        <x:v>163</x:v>
+      </x:c>
+      <x:c r="F167" s="30" t="str">
+        <x:v>13.2</x:v>
+      </x:c>
+      <x:c r="G167" s="30" t="str">
+        <x:v>Eigene Restaurantseite mit Atmosphäre, Angebot, Lage, Reservationshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H167" s="30" t="str">
+        <x:v>Platzhalter</x:v>
+      </x:c>
+      <x:c r="I167" s="30" t="str">
+        <x:v>platzhalter.png, bis ein lizenziertes Bild vorliegt</x:v>
+      </x:c>
+      <x:c r="J167" s="30" t="str">
+        <x:v>Kachel / Link bei Restaurants</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="168">
+      <x:c r="A168" s="30" t="str">
+        <x:v>Übernachten</x:v>
+      </x:c>
+      <x:c r="B168" s="30" t="str">
+        <x:v>Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+      <x:c r="C168" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D168" s="30" t="str">
+        <x:v>1740 Boutique Hotel Kazbegi</x:v>
+      </x:c>
+      <x:c r="E168" s="39" t="n">
+        <x:v>164</x:v>
+      </x:c>
+      <x:c r="F168" s="30" t="str">
+        <x:v>13.1</x:v>
+      </x:c>
+      <x:c r="G168" s="30" t="str">
+        <x:v>Eigene Unterkunftsseite mit Lage, Charakter, Zimmern, Buchungshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H168" s="30" t="str">
+        <x:v>Platzhalter</x:v>
+      </x:c>
+      <x:c r="I168" s="30" t="str">
+        <x:v>platzhalter.png, bis ein lizenziertes Bild vorliegt</x:v>
+      </x:c>
+      <x:c r="J168" s="30" t="str">
+        <x:v>Kachel / Link bei Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169">
+      <x:c r="A169" s="30" t="str">
+        <x:v>Übernachten</x:v>
+      </x:c>
+      <x:c r="B169" s="30" t="str">
+        <x:v>Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+      <x:c r="C169" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D169" s="30" t="str">
+        <x:v>Castello Mare Hotel &amp; Wellness Resort</x:v>
+      </x:c>
+      <x:c r="E169" s="39" t="n">
+        <x:v>165</x:v>
+      </x:c>
+      <x:c r="F169" s="30" t="str">
+        <x:v>13.1</x:v>
+      </x:c>
+      <x:c r="G169" s="30" t="str">
+        <x:v>Eigene Unterkunftsseite mit Lage, Charakter, Zimmern, Buchungshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H169" s="30" t="str">
+        <x:v>Platzhalter</x:v>
+      </x:c>
+      <x:c r="I169" s="30" t="str">
+        <x:v>platzhalter.png, bis ein lizenziertes Bild vorliegt</x:v>
+      </x:c>
+      <x:c r="J169" s="30" t="str">
+        <x:v>Kachel / Link bei Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="170">
+      <x:c r="A170" s="30" t="str">
+        <x:v>Übernachten</x:v>
+      </x:c>
+      <x:c r="B170" s="30" t="str">
+        <x:v>Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+      <x:c r="C170" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D170" s="30" t="str">
+        <x:v>EL Hotel</x:v>
+      </x:c>
+      <x:c r="E170" s="39" t="n">
+        <x:v>166</x:v>
+      </x:c>
+      <x:c r="F170" s="30" t="str">
+        <x:v>13.1</x:v>
+      </x:c>
+      <x:c r="G170" s="30" t="str">
+        <x:v>Eigene Unterkunftsseite mit Lage, Charakter, Zimmern, Buchungshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H170" s="30" t="str">
+        <x:v>Platzhalter</x:v>
+      </x:c>
+      <x:c r="I170" s="30" t="str">
+        <x:v>platzhalter.png, bis ein lizenziertes Bild vorliegt</x:v>
+      </x:c>
+      <x:c r="J170" s="30" t="str">
+        <x:v>Kachel / Link bei Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="171">
+      <x:c r="A171" s="30" t="str">
+        <x:v>Übernachten</x:v>
+      </x:c>
+      <x:c r="B171" s="30" t="str">
+        <x:v>Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+      <x:c r="C171" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D171" s="30" t="str">
+        <x:v>Georgia Palace Hotel &amp; Spa</x:v>
+      </x:c>
+      <x:c r="E171" s="39" t="n">
+        <x:v>167</x:v>
+      </x:c>
+      <x:c r="F171" s="30" t="str">
+        <x:v>13.1</x:v>
+      </x:c>
+      <x:c r="G171" s="30" t="str">
+        <x:v>Eigene Unterkunftsseite mit Lage, Charakter, Zimmern, Buchungshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H171" s="30" t="str">
+        <x:v>Platzhalter</x:v>
+      </x:c>
+      <x:c r="I171" s="30" t="str">
+        <x:v>platzhalter.png, bis ein lizenziertes Bild vorliegt</x:v>
+      </x:c>
+      <x:c r="J171" s="30" t="str">
+        <x:v>Kachel / Link bei Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="172">
+      <x:c r="A172" s="30" t="str">
+        <x:v>Übernachten</x:v>
+      </x:c>
+      <x:c r="B172" s="30" t="str">
+        <x:v>Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+      <x:c r="C172" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D172" s="30" t="str">
+        <x:v>Hotel Pavo</x:v>
+      </x:c>
+      <x:c r="E172" s="39" t="n">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="F172" s="30" t="str">
+        <x:v>13.1</x:v>
+      </x:c>
+      <x:c r="G172" s="30" t="str">
+        <x:v>Eigene Unterkunftsseite mit Lage, Charakter, Zimmern, Buchungshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H172" s="30" t="str">
+        <x:v>Platzhalter</x:v>
+      </x:c>
+      <x:c r="I172" s="30" t="str">
+        <x:v>platzhalter.png, bis ein lizenziertes Bild vorliegt</x:v>
+      </x:c>
+      <x:c r="J172" s="30" t="str">
+        <x:v>Kachel / Link bei Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="173">
+      <x:c r="A173" s="30" t="str">
+        <x:v>Übernachten</x:v>
+      </x:c>
+      <x:c r="B173" s="30" t="str">
+        <x:v>Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+      <x:c r="C173" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D173" s="30" t="str">
+        <x:v>Magnetic Resort Ureki</x:v>
+      </x:c>
+      <x:c r="E173" s="39" t="n">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="F173" s="30" t="str">
+        <x:v>13.1</x:v>
+      </x:c>
+      <x:c r="G173" s="30" t="str">
+        <x:v>Eigene Unterkunftsseite mit Lage, Charakter, Zimmern, Buchungshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H173" s="30" t="str">
+        <x:v>Platzhalter</x:v>
+      </x:c>
+      <x:c r="I173" s="30" t="str">
+        <x:v>platzhalter.png, bis ein lizenziertes Bild vorliegt</x:v>
+      </x:c>
+      <x:c r="J173" s="30" t="str">
+        <x:v>Kachel / Link bei Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="174">
+      <x:c r="A174" s="30" t="str">
+        <x:v>Übernachten</x:v>
+      </x:c>
+      <x:c r="B174" s="30" t="str">
+        <x:v>Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+      <x:c r="C174" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D174" s="30" t="str">
+        <x:v>Miramare Magnetic Beach Hotel</x:v>
+      </x:c>
+      <x:c r="E174" s="39" t="n">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="F174" s="30" t="str">
+        <x:v>13.1</x:v>
+      </x:c>
+      <x:c r="G174" s="30" t="str">
+        <x:v>Eigene Unterkunftsseite mit Lage, Charakter, Zimmern, Buchungshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H174" s="30" t="str">
+        <x:v>Platzhalter</x:v>
+      </x:c>
+      <x:c r="I174" s="30" t="str">
+        <x:v>platzhalter.png, bis ein lizenziertes Bild vorliegt</x:v>
+      </x:c>
+      <x:c r="J174" s="30" t="str">
+        <x:v>Kachel / Link bei Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="175">
+      <x:c r="A175" s="30" t="str">
+        <x:v>Übernachten</x:v>
+      </x:c>
+      <x:c r="B175" s="30" t="str">
+        <x:v>Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+      <x:c r="C175" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D175" s="30" t="str">
+        <x:v>Newport Hotel Kutaisi</x:v>
+      </x:c>
+      <x:c r="E175" s="39" t="n">
+        <x:v>171</x:v>
+      </x:c>
+      <x:c r="F175" s="30" t="str">
+        <x:v>13.1</x:v>
+      </x:c>
+      <x:c r="G175" s="30" t="str">
+        <x:v>Eigene Unterkunftsseite mit Lage, Charakter, Zimmern, Buchungshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H175" s="30" t="str">
+        <x:v>Platzhalter</x:v>
+      </x:c>
+      <x:c r="I175" s="30" t="str">
+        <x:v>platzhalter.png, bis ein lizenziertes Bild vorliegt</x:v>
+      </x:c>
+      <x:c r="J175" s="30" t="str">
+        <x:v>Kachel / Link bei Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="176">
+      <x:c r="A176" s="30" t="str">
+        <x:v>Übernachten</x:v>
+      </x:c>
+      <x:c r="B176" s="30" t="str">
+        <x:v>Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+      <x:c r="C176" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D176" s="30" t="str">
+        <x:v>Old Town Mtatsminda</x:v>
+      </x:c>
+      <x:c r="E176" s="39" t="n">
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="F176" s="30" t="str">
+        <x:v>13.1</x:v>
+      </x:c>
+      <x:c r="G176" s="30" t="str">
+        <x:v>Eigene Unterkunftsseite mit Lage, Charakter, Zimmern, Buchungshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H176" s="30" t="str">
+        <x:v>Platzhalter</x:v>
+      </x:c>
+      <x:c r="I176" s="30" t="str">
+        <x:v>platzhalter.png, bis ein lizenziertes Bild vorliegt</x:v>
+      </x:c>
+      <x:c r="J176" s="30" t="str">
+        <x:v>Kachel / Link bei Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="177">
+      <x:c r="A177" s="30" t="str">
+        <x:v>Übernachten</x:v>
+      </x:c>
+      <x:c r="B177" s="30" t="str">
+        <x:v>Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+      <x:c r="C177" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D177" s="30" t="str">
+        <x:v>Paragraph Resort &amp; Spa</x:v>
+      </x:c>
+      <x:c r="E177" s="39" t="n">
+        <x:v>173</x:v>
+      </x:c>
+      <x:c r="F177" s="30" t="str">
+        <x:v>13.1</x:v>
+      </x:c>
+      <x:c r="G177" s="30" t="str">
+        <x:v>Eigene Unterkunftsseite mit Lage, Charakter, Zimmern, Buchungshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H177" s="30" t="str">
+        <x:v>Platzhalter</x:v>
+      </x:c>
+      <x:c r="I177" s="30" t="str">
+        <x:v>platzhalter.png, bis ein lizenziertes Bild vorliegt</x:v>
+      </x:c>
+      <x:c r="J177" s="30" t="str">
+        <x:v>Kachel / Link bei Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="178">
+      <x:c r="A178" s="30" t="str">
+        <x:v>Übernachten</x:v>
+      </x:c>
+      <x:c r="B178" s="30" t="str">
+        <x:v>Hotels &amp; Unterkünfte</x:v>
+      </x:c>
+      <x:c r="C178" s="30" t="str">
+        <x:v>Detailseite</x:v>
+      </x:c>
+      <x:c r="D178" s="30" t="str">
+        <x:v>Rooms Hotel Kazbegi</x:v>
+      </x:c>
+      <x:c r="E178" s="39" t="n">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="F178" s="30" t="str">
+        <x:v>13.1</x:v>
+      </x:c>
+      <x:c r="G178" s="30" t="str">
+        <x:v>Eigene Unterkunftsseite mit Lage, Charakter, Zimmern, Buchungshinweisen und Bezug zur Route.</x:v>
+      </x:c>
+      <x:c r="H178" s="30" t="str">
+        <x:v>Platzhalter</x:v>
+      </x:c>
+      <x:c r="I178" s="30" t="str">
+        <x:v>platzhalter.png, bis ein lizenziertes Bild vorliegt</x:v>
+      </x:c>
+      <x:c r="J178" s="30" t="str">
+        <x:v>Kachel / Link bei Hotels &amp; Unterkünfte</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -8347,7 +8926,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0960ab9c1ae1452d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R202fb6294de44b71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>